<commit_message>
fix(unit02): repair lesson and practice integrity
</commit_message>
<xml_diff>
--- a/bus-math-nextjs/public/resources/unit02-lesson05-teacher.xlsx
+++ b/bus-math-nextjs/public/resources/unit02-lesson05-teacher.xlsx
@@ -79,7 +79,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -92,11 +92,20 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -109,6 +118,7 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -505,6 +515,9 @@
           <t>TechStart Month-End Adjustment Inputs</t>
         </is>
       </c>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -547,7 +560,6 @@
       <c r="C5" s="4" t="n">
         <v>5500</v>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -561,7 +573,6 @@
       <c r="C6" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -575,7 +586,6 @@
       <c r="C7" s="4" t="n">
         <v>2000</v>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -589,7 +599,6 @@
       <c r="C8" s="4" t="n">
         <v>4000</v>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -603,7 +612,6 @@
       <c r="C9" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -646,6 +654,12 @@
           <t>TechStart Month-End Close Model</t>
         </is>
       </c>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
+      <c r="E1" s="8" t="n"/>
+      <c r="F1" s="8" t="n"/>
+      <c r="G1" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1344,6 +1358,7 @@
           <t>Month-End Close Control Panel</t>
         </is>
       </c>
+      <c r="B1" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1418,7 +1433,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(AND(B6=0,B7=0,B8=0),"Complete","Review flagged items")</f>
+        <f>IF(OR(COUNT('Close Model'!B4:C13)&lt;&gt;20,COUNT('Close Model'!F19:G33)&lt;&gt;30),"Not finished",IF(AND(B6=0,B7=0,B8=0),"Complete","Review flagged items"))</f>
         <v/>
       </c>
     </row>

</xml_diff>